<commit_message>
docs(acquire): set asking price to 4,500 USD with explicit numeric /bin/bash.00 TTM totals per Harold Ecoy
</commit_message>
<xml_diff>
--- a/GRANTS/evidence/FactLedger_PnL_and_Valuation_2026.xlsx
+++ b/GRANTS/evidence/FactLedger_PnL_and_Valuation_2026.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TTM_PnL_Statement" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commercial_Model_and_Valuation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Summary_24500_Buyout" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -49,19 +48,19 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001E293B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00B45309"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -119,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,20 +129,26 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -509,10 +514,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -538,7 +543,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Owner: Abdullah Al-Anzi (100% Bootstrapped IP) | Currency: USD | Basis: Cash / Actuals (Nov 2025 – Oct 2026)</t>
+          <t>Owner: Abdullah Al-Anzi | Asking Price: $24,500 USD (Pre-Revenue SaaS) | Basis: Actuals (Nov 2025 – Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -637,7 +642,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>SaaS API &amp; MCP Subscriptions (Launched Oct 2026)</t>
+          <t>SaaS API &amp; MCP Subscriptions</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
@@ -676,15 +681,14 @@
       <c r="M6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="8">
-        <f>SUM(B6:M6)</f>
-        <v/>
+      <c r="N6" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Institutional Audit Reports (100-Report Catalog)</t>
+          <t>Institutional Audit Reports</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -723,9 +727,8 @@
       <c r="M7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="8">
-        <f>SUM(B7:M7)</f>
-        <v/>
+      <c r="N7" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -770,9 +773,8 @@
       <c r="M8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="8">
-        <f>SUM(B8:M8)</f>
-        <v/>
+      <c r="N8" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -781,63 +783,50 @@
           <t>Total Gross Revenue (TTM)</t>
         </is>
       </c>
-      <c r="B9" s="10">
-        <f>SUM(B6:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="10">
-        <f>SUM(C6:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="10">
-        <f>SUM(D6:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="10">
-        <f>SUM(E6:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="10">
-        <f>SUM(F6:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="10">
-        <f>SUM(G6:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="10">
-        <f>SUM(H6:H8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="10">
-        <f>SUM(I6:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="10">
-        <f>SUM(J6:J8)</f>
-        <v/>
-      </c>
-      <c r="K9" s="10">
-        <f>SUM(K6:K8)</f>
-        <v/>
-      </c>
-      <c r="L9" s="10">
-        <f>SUM(L6:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="10">
-        <f>SUM(M6:M8)</f>
-        <v/>
-      </c>
-      <c r="N9" s="10">
-        <f>SUM(B9:M9)</f>
-        <v/>
+      <c r="B9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>OPERATING EXPENSES (CLOUD &amp; INFRASTRUCTURE)</t>
+          <t>COST OF GOODS SOLD (COGS)</t>
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
@@ -857,7 +846,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Cloud Hosting (Render API &amp; Demo Free/Starter Tier)</t>
+          <t>Cloud Hosting (Render Free/Starter Tier)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -896,15 +885,14 @@
       <c r="M11" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="8">
-        <f>SUM(B11:M11)</f>
-        <v/>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Solana Mainnet RPC &amp; Telemetry (Public / Open Tier)</t>
+          <t>Solana Mainnet RPC &amp; Telemetry (Public Tier)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -943,221 +931,417 @@
       <c r="M12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="8">
-        <f>SUM(B12:M12)</f>
-        <v/>
+      <c r="N12" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>GitHub Actions CI/CD &amp; CodeQL Security (Open-Source Tier)</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="8">
-        <f>SUM(B13:M13)</f>
-        <v/>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Total COGS (TTM)</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Founder R&amp;D / Engineering (100% Founder Sweat Equity)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="8">
-        <f>SUM(B14:M14)</f>
-        <v/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>GROSS PROFIT (TTM)</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>OPERATING EXPENSES (OPEX)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI/CD &amp; Security (Open-Source Tier)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>General &amp; Administrative / R&amp;D (100% Founder Sweat Equity)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Total Operating Expenses (TTM)</t>
         </is>
       </c>
-      <c r="B15" s="11">
-        <f>SUM(B11:B14)</f>
-        <v/>
-      </c>
-      <c r="C15" s="11">
-        <f>SUM(C11:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="11">
-        <f>SUM(D11:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="11">
-        <f>SUM(E11:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="11">
-        <f>SUM(F11:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="11">
-        <f>SUM(G11:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="11">
-        <f>SUM(H11:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="11">
-        <f>SUM(I11:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="11">
-        <f>SUM(J11:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="11">
-        <f>SUM(K11:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="11">
-        <f>SUM(L11:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="11">
-        <f>SUM(M11:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="11">
-        <f>SUM(B15:M15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>NET PROFIT / EBITDA (TTM ACTUAL)</t>
-        </is>
-      </c>
-      <c r="B16" s="10">
-        <f>B9-B15</f>
-        <v/>
-      </c>
-      <c r="C16" s="10">
-        <f>C9-C15</f>
-        <v/>
-      </c>
-      <c r="D16" s="10">
-        <f>D9-D15</f>
-        <v/>
-      </c>
-      <c r="E16" s="10">
-        <f>E9-E15</f>
-        <v/>
-      </c>
-      <c r="F16" s="10">
-        <f>F9-F15</f>
-        <v/>
-      </c>
-      <c r="G16" s="10">
-        <f>G9-G15</f>
-        <v/>
-      </c>
-      <c r="H16" s="10">
-        <f>H9-H15</f>
-        <v/>
-      </c>
-      <c r="I16" s="10">
-        <f>I9-I15</f>
-        <v/>
-      </c>
-      <c r="J16" s="10">
-        <f>J9-J15</f>
-        <v/>
-      </c>
-      <c r="K16" s="10">
-        <f>K9-K15</f>
-        <v/>
-      </c>
-      <c r="L16" s="10">
-        <f>L9-L15</f>
-        <v/>
-      </c>
-      <c r="M16" s="10">
-        <f>M9-M15</f>
-        <v/>
-      </c>
-      <c r="N16" s="10">
-        <f>N9-N15</f>
-        <v/>
+      <c r="B19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>NET PROFIT / SDE / EBITDA (TTM ACTUAL)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>ACQUIRE.COM LISTING FINANCIAL SUMMARY (COMPLETED NUMERIC TOTALS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Trailing 12-Month (TTM) Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Trailing 12-Month (TTM) Total Expenses</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Trailing 12-Month (TTM) Net Profit / SDE</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Last Month Gross Revenue (Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Last Month Net Profit (Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Asking Price (Pre-Revenue SaaS Criteria &lt; $25,000)</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>24500</v>
       </c>
     </row>
   </sheetData>
@@ -1171,10 +1355,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1193,230 +1377,110 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FACTLEDGER — COMMERCIAL MONETIZATION SCHEDULE &amp; ACQUISITION VALUATION</t>
+          <t>FACTLEDGER — PRE-REVENUE SAAS ASSET SUMMARY ($24,500 USD ASKING PRICE)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Note: The $75,000 and $150,000 figures previously entered in the draft form represented forward annualized projections &amp; asking valuation, not trailing TTM actuals.</t>
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Compliant with Acquire.com Pre-Revenue SaaS Criteria (&lt; $25,000 Asking Price | $0 TTM Revenue | $0 TTM Profit)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Revenue Stream / Asset Tier</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Unit Price (USD)</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>Target Monthly Volume</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Projected Monthly Revenue (MRR)</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>Projected Annual Run Rate (ARR)</t>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Listing Asking Price (Cash at Close)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>$24,500.00 USD</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Pro Developer &amp; AI Agent API/MCP Plan (25k req/mo)</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="n">
-        <v>149</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" s="8">
-        <f>B5*C5</f>
-        <v/>
-      </c>
-      <c r="E5" s="8">
-        <f>D5*12</f>
-        <v/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>TTM Revenue (Actual Historical)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>$0.00 USD</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Business Protocol &amp; Wallet Plan (250k req/mo + 10 alert streams)</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>499</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" s="8">
-        <f>B6*C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="8">
-        <f>D6*12</f>
-        <v/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TTM Net Profit (Actual Historical)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$0.00 USD</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Institutional Wallet/Protocol Audit Reports (100-Report Engine)</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>500</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="D7" s="8">
-        <f>B7*C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="8">
-        <f>D7*12</f>
-        <v/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Last Month Profit (Actual Historical)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$0.00 USD</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>On-Chain Pay-Per-Scan Micropayments (MicropaymentVerifier)</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>3500</v>
-      </c>
-      <c r="D8" s="8">
-        <f>B8*C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="8">
-        <f>D8*12</f>
-        <v/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Codebase &amp; Test Suite</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>TypeScript Strict Mode • 224 Automated CI Tests Passing (100%)</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Ecosystem Grants &amp; Sponsorships (Solana / Pyth / Superteam)</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8">
-        <f>B9*C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="8">
-        <f>D9*12</f>
-        <v/>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>AI &amp; Agent Layer</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>8-Tool Model Context Protocol (MCP) Server + 100-Agent Verification Suite</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL PROJECTED COMMERCIAL CAPACITY</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr"/>
-      <c r="C10" s="18" t="inlineStr"/>
-      <c r="D10" s="10">
-        <f>SUM(D5:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="10">
-        <f>SUM(E5:E9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>ACQUISITION ASKING PRICE &amp; ASSET SUMMARY (100% IP &amp; CODEBASE BUYOUT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Corrected Trailing 12-Month (TTM) Revenue</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>$0 (Pre-Revenue / Newly Launched Commercial Asset)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Corrected Trailing 12-Month (TTM) Net Profit</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>$0 (Zero Debt, Zero External Liabilities)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Corrected Last Month Profit</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Target Cash Acquisition Asking Price</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>$75,000 USD (Open to Cash Offers from $35,000 - $75,000 USD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Included Technical Assets</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>TypeScript Core (224 CI Tests), 8-Tool MCP Server, 100-Agent Verification Suite, 100-Report Engine, Live Render API &amp; Demo</t>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Institutional Reports Engine</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>100 Deterministic Solana Audit Reports Catalog (RPT-001 to RPT-100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Built-in Monetization Tiers</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Free (1k req) | Pro ($149/mo) | Business ($499/mo) | Enterprise ($1,500/mo) + On-Chain SOL Micropayments</t>
         </is>
       </c>
     </row>

</xml_diff>